<commit_message>
Add KRONOS per-class AP reference column to CODEX_cHL_KRONOS18_AP sheet
Adds KRONOS_AP dict (Table S7, arXiv:2506.03373) with 16 cell-type AP
values (mean over 4 folds) as a reference column alongside our 4 models.
MEAN row confirms CIM_Funnel_Large (0.7605) matches KRONOS (0.7614).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/paper_results.xlsx
+++ b/paper_results.xlsx
@@ -1499,7 +1499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1507,6 +1507,7 @@
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1535,6 +1536,11 @@
           <t>ResNet</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>KRONOS</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1562,6 +1568,11 @@
           <t>0.7640</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0.7927</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1589,6 +1600,11 @@
           <t>0.7332</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0.8369</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1616,6 +1632,11 @@
           <t>0.8073</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>0.9089</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1643,6 +1664,11 @@
           <t>0.6345</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>0.6817</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1670,6 +1696,11 @@
           <t>0.7982</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>0.8473</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1697,6 +1728,11 @@
           <t>0.0437</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>0.6186</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1724,6 +1760,11 @@
           <t>0.7697</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>0.9053</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1751,6 +1792,11 @@
           <t>0.5083</t>
         </is>
       </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>0.5368</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1778,6 +1824,11 @@
           <t>0.6679</t>
         </is>
       </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>0.7317</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1805,6 +1856,11 @@
           <t>0.2426</t>
         </is>
       </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>0.8357</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1832,6 +1888,11 @@
           <t>0.3850</t>
         </is>
       </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>0.5737</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1859,6 +1920,11 @@
           <t>0.6065</t>
         </is>
       </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>0.7747</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1886,6 +1952,11 @@
           <t>0.7554</t>
         </is>
       </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>0.7505</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1913,6 +1984,11 @@
           <t>0.5041</t>
         </is>
       </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>0.6458</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1940,6 +2016,11 @@
           <t>0.2446</t>
         </is>
       </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>0.8150</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1967,6 +2048,11 @@
           <t>0.9119</t>
         </is>
       </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>0.9267</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1992,6 +2078,11 @@
       <c r="E18" t="inlineStr">
         <is>
           <t>0.5861</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>0.7614</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ExprBaseline + DINOv2/UNI/OpenPhenom to Excel summary and AP sheets
make_paper_excel.py now runs locally, loading paper_clean results from
synced z_RUNS/paper_clean/ and external model results from z_RUNS/.
Handles two metrics.json formats (old flat val/ and new nested
linear_probe/knn/ format). Applies annotation_map normalisation
(Cytotoxic CD8→CD8, TReg→Treg) and drops Seg Artifact/Unidentified
before merging class-level AP across all models.

All summary sheets now include ExprBaseline, DINOv2, OpenPhenom, UNI
rows; all _AP sheets gain those as additional columns (+ KRONOS for
CODEX_cHL_KRONOS18).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/paper_results.xlsx
+++ b/paper_results.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -695,6 +695,162 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ExprBaseline</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>16</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>0.6601</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>0.6298</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>0.6643</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>0.5111</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>0.2568</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>0.0901</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>DINOv2</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>16</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>0.1963</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>0.1700</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>0.0869</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>0.0133</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>0.0047</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>OpenPhenom</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>16</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>0.2229</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>0.1781</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>0.1195</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>0.0371</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>0.0126</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>UNI</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>16</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>0.2512</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>0.2119</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>0.1142</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>0.0262</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>0.0096</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -706,7 +862,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -714,6 +870,10 @@
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -742,6 +902,26 @@
           <t>ResNet</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>ExprBaseline</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>DINOv2</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>OpenPhenom</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>UNI</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -769,6 +949,26 @@
           <t>0.7690</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0.7392</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0.2436</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>0.2343</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>0.2959</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -796,6 +996,26 @@
           <t>0.7619</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0.7947</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0.3683</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>0.3737</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>0.4011</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -823,6 +1043,26 @@
           <t>0.8006</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>0.6531</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>0.1082</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>0.1189</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>0.1345</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -850,6 +1090,26 @@
           <t>0.6440</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>0.6365</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>0.1107</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>0.1337</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>0.1722</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -877,6 +1137,26 @@
           <t>0.7987</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>0.8461</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>0.2536</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>0.1922</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>0.3193</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -904,6 +1184,26 @@
           <t>0.0843</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>0.1006</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>0.0270</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>0.0430</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>0.0452</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -931,6 +1231,26 @@
           <t>0.6895</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>0.8761</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>0.0565</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>0.0615</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>0.0733</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -958,6 +1278,26 @@
           <t>0.5121</t>
         </is>
       </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>0.5342</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>0.0356</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>0.0360</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>0.0449</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -985,6 +1325,26 @@
           <t>0.6919</t>
         </is>
       </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>0.7291</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>0.0986</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>0.1206</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>0.1286</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1012,6 +1372,26 @@
           <t>0.7555</t>
         </is>
       </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>0.8386</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>0.0488</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>0.0494</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>0.0668</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1039,6 +1419,26 @@
           <t>0.3832</t>
         </is>
       </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>0.4506</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>0.3026</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>0.2815</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>0.3302</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1066,6 +1466,26 @@
           <t>0.6033</t>
         </is>
       </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>0.6818</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>0.3012</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>0.3492</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>0.3762</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1093,6 +1513,26 @@
           <t>0.7602</t>
         </is>
       </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>0.7838</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>0.0559</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>0.0629</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>0.0803</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1120,6 +1560,26 @@
           <t>0.5205</t>
         </is>
       </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>0.6213</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>0.2356</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>0.2875</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>0.3272</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1147,6 +1607,26 @@
           <t>0.4307</t>
         </is>
       </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>0.4184</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>0.0488</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>0.0941</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>0.0770</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1174,6 +1654,26 @@
           <t>0.9185</t>
         </is>
       </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>0.9248</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>0.4255</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>0.4110</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>0.5182</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1199,6 +1699,26 @@
       <c r="E18" t="inlineStr">
         <is>
           <t>0.6327</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>0.6643</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>0.1700</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>0.1781</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>0.2119</t>
         </is>
       </c>
     </row>
@@ -2097,7 +2617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -2372,6 +2892,162 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ExprBaseline</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>16</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>0.7400</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>0.7586</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>0.6617</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>0.5322</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>0.2042</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>0.0672</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>DINOv2</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>16</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>0.2563</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>0.1695</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>0.0875</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>0.0308</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>0.0094</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>OpenPhenom</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>16</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>0.2723</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>0.1699</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>0.1094</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>0.1050</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>0.0355</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>UNI</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>16</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>0.3139</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>0.2152</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>0.1112</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>0.0533</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>0.0090</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2383,7 +3059,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -2391,6 +3067,10 @@
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2419,6 +3099,26 @@
           <t>ResNet</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>ExprBaseline</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>DINOv2</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>OpenPhenom</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>UNI</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2446,6 +3146,26 @@
           <t>0.7845</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0.8812</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0.3611</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>0.2699</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>0.4604</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2473,6 +3193,26 @@
           <t>0.3747</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0.6105</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0.0537</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>0.0625</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>0.0913</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2500,6 +3240,26 @@
           <t>0.7296</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>0.8776</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>0.2747</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>0.2520</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>0.3323</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2527,6 +3287,26 @@
           <t>0.8700</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>0.9450</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>0.2073</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>0.2281</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>0.2386</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2554,6 +3334,26 @@
           <t>0.0157</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>0.7388</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>0.0228</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>0.0373</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>0.0746</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2581,6 +3381,26 @@
           <t>0.3448</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>0.5026</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>0.0591</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>0.0547</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>0.0763</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2608,6 +3428,26 @@
           <t>0.2854</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>0.3686</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>0.0324</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>0.0363</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>0.0567</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2635,6 +3475,26 @@
           <t>0.9745</t>
         </is>
       </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>0.9819</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>0.8158</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>0.8128</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>0.8517</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2662,6 +3522,26 @@
           <t>0.6526</t>
         </is>
       </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>0.8557</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>0.2361</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>0.2385</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>0.2772</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2689,6 +3569,26 @@
           <t>0.4428</t>
         </is>
       </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>0.4836</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>0.2183</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>0.1996</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>0.2744</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2716,6 +3616,26 @@
           <t>0.1466</t>
         </is>
       </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>0.2750</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>0.0427</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>0.0491</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>0.0610</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2743,6 +3663,26 @@
           <t>0.0314</t>
         </is>
       </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>0.5935</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>0.0101</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>0.0124</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>0.0101</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2770,6 +3710,26 @@
           <t>0.3289</t>
         </is>
       </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>0.7784</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>0.0506</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>0.0374</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>0.0745</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2797,6 +3757,26 @@
           <t>0.3956</t>
         </is>
       </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>0.6050</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>0.1300</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>0.1316</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>0.2159</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2824,6 +3804,26 @@
           <t>0.2757</t>
         </is>
       </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>0.8564</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>0.0713</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>0.0872</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>0.1475</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2851,6 +3851,26 @@
           <t>0.1547</t>
         </is>
       </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>0.2327</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>0.1261</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>0.2097</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>0.2003</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2876,6 +3896,26 @@
       <c r="E18" t="inlineStr">
         <is>
           <t>0.4255</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>0.6617</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>0.1695</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>0.1699</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>0.2152</t>
         </is>
       </c>
     </row>
@@ -2890,7 +3930,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -3165,6 +4205,120 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>DINOv2</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>20</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>0.1837</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>0.1524</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>0.1203</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>0.0624</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>0.0205</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>OpenPhenom</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>20</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>0.1620</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>0.1326</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>0.1357</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>0.1003</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>0.0379</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>UNI</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>20</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>0.1994</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>0.1634</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>0.1284</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>0.0712</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>0.0216</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3176,7 +4330,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3184,6 +4338,9 @@
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3212,6 +4369,21 @@
           <t>ResNet</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>DINOv2</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>OpenPhenom</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>UNI</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3239,6 +4411,21 @@
           <t>0.6991</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0.1006</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0.1264</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>0.1430</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3266,6 +4453,21 @@
           <t>0.5520</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0.0130</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0.0139</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>0.0131</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3293,6 +4495,21 @@
           <t>0.7772</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>0.0256</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>0.0240</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>0.0235</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3320,6 +4537,21 @@
           <t>0.7348</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>0.0392</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>0.0381</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>0.0392</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3347,6 +4579,21 @@
           <t>0.0836</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>0.0005</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>0.0006</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>0.0006</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3374,6 +4621,21 @@
           <t>0.5255</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>0.0463</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>0.0515</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>0.0611</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3401,6 +4663,21 @@
           <t>0.4743</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>0.0237</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>0.0214</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>0.0289</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3428,6 +4705,21 @@
           <t>0.8487</t>
         </is>
       </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>0.2260</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>0.2227</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>0.2546</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3455,6 +4747,21 @@
           <t>0.9213</t>
         </is>
       </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>0.2280</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>0.2013</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>0.2410</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3482,6 +4789,21 @@
           <t>0.7559</t>
         </is>
       </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>0.5340</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>0.4488</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>0.5436</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3509,6 +4831,21 @@
           <t>0.5876</t>
         </is>
       </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>0.2060</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>0.1686</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>0.2190</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3536,6 +4873,21 @@
           <t>0.8247</t>
         </is>
       </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>0.3404</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>0.3296</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>0.3483</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3563,6 +4915,21 @@
           <t>0.1804</t>
         </is>
       </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>0.0044</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>0.0042</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>0.0039</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3590,6 +4957,21 @@
           <t>0.7860</t>
         </is>
       </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>0.2714</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>0.2421</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>0.2923</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3617,6 +4999,21 @@
           <t>0.1679</t>
         </is>
       </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>0.0117</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>0.0106</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>0.0140</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3644,6 +5041,21 @@
           <t>0.2530</t>
         </is>
       </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>0.0508</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>0.0408</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>0.0607</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3671,6 +5083,21 @@
           <t>0.7243</t>
         </is>
       </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>0.1965</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>0.1702</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>0.2078</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3698,6 +5125,21 @@
           <t>0.8149</t>
         </is>
       </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>0.3016</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>0.2796</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>0.3113</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3725,6 +5167,21 @@
           <t>0.7349</t>
         </is>
       </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>0.1888</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>0.1564</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>0.2165</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3750,6 +5207,21 @@
       <c r="E21" t="inlineStr">
         <is>
           <t>0.6024</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>0.1524</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>0.1326</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>0.1634</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove DINOv2/UNI/OpenPhenom columns from Excel — keep ExprBaseline only
Foundation models perform at near-chance on multiplexed imaging data
and need to be reassessed before inclusion in the paper comparison.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/paper_results.xlsx
+++ b/paper_results.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -737,120 +737,6 @@
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>DINOv2</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>16</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>0.1963</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>0.1700</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>0.0869</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>0.0133</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>0.0047</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>OpenPhenom</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>16</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>0.2229</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>0.1781</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>0.1195</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>0.0371</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>0.0126</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>UNI</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>16</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>0.2512</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>0.2119</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>0.1142</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>0.0262</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>0.0096</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -862,7 +748,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -871,9 +757,6 @@
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -907,21 +790,6 @@
           <t>ExprBaseline</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>DINOv2</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>OpenPhenom</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>UNI</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -954,21 +822,6 @@
           <t>0.7392</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>0.2436</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>0.2343</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>0.2959</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1001,21 +854,6 @@
           <t>0.7947</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>0.3683</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>0.3737</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>0.4011</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1048,21 +886,6 @@
           <t>0.6531</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>0.1082</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>0.1189</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>0.1345</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1095,21 +918,6 @@
           <t>0.6365</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>0.1107</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>0.1337</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>0.1722</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1142,21 +950,6 @@
           <t>0.8461</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>0.2536</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>0.1922</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>0.3193</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1189,21 +982,6 @@
           <t>0.1006</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>0.0270</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>0.0430</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>0.0452</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1236,21 +1014,6 @@
           <t>0.8761</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>0.0565</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>0.0615</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>0.0733</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1283,21 +1046,6 @@
           <t>0.5342</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>0.0356</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>0.0360</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>0.0449</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1330,21 +1078,6 @@
           <t>0.7291</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>0.0986</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>0.1206</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>0.1286</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1377,21 +1110,6 @@
           <t>0.8386</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>0.0488</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>0.0494</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>0.0668</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1424,21 +1142,6 @@
           <t>0.4506</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>0.3026</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>0.2815</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>0.3302</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1471,21 +1174,6 @@
           <t>0.6818</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>0.3012</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>0.3492</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>0.3762</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1518,21 +1206,6 @@
           <t>0.7838</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>0.0559</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>0.0629</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>0.0803</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1565,21 +1238,6 @@
           <t>0.6213</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>0.2356</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>0.2875</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>0.3272</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1612,21 +1270,6 @@
           <t>0.4184</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>0.0488</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>0.0941</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>0.0770</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1659,21 +1302,6 @@
           <t>0.9248</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>0.4255</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>0.4110</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>0.5182</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1704,21 +1332,6 @@
       <c r="F18" t="inlineStr">
         <is>
           <t>0.6643</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>0.1700</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>0.1781</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>0.2119</t>
         </is>
       </c>
     </row>
@@ -2617,7 +2230,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -2934,120 +2547,6 @@
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>DINOv2</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>16</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>0.2563</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>0.1695</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>0.0875</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>0.0308</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>0.0094</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>OpenPhenom</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>16</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>0.2723</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>0.1699</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>0.1094</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>0.1050</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>0.0355</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>UNI</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>16</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>0.3139</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>0.2152</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>0.1112</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>0.0533</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>0.0090</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3059,7 +2558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -3068,9 +2567,6 @@
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3104,21 +2600,6 @@
           <t>ExprBaseline</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>DINOv2</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>OpenPhenom</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>UNI</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3151,21 +2632,6 @@
           <t>0.8812</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>0.3611</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>0.2699</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>0.4604</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3198,21 +2664,6 @@
           <t>0.6105</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>0.0537</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>0.0625</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>0.0913</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3245,21 +2696,6 @@
           <t>0.8776</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>0.2747</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>0.2520</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>0.3323</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3292,21 +2728,6 @@
           <t>0.9450</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>0.2073</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>0.2281</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>0.2386</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3339,21 +2760,6 @@
           <t>0.7388</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>0.0228</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>0.0373</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>0.0746</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3386,21 +2792,6 @@
           <t>0.5026</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>0.0591</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>0.0547</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>0.0763</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3433,21 +2824,6 @@
           <t>0.3686</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>0.0324</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>0.0363</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>0.0567</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3480,21 +2856,6 @@
           <t>0.9819</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>0.8158</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>0.8128</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>0.8517</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3527,21 +2888,6 @@
           <t>0.8557</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>0.2361</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>0.2385</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>0.2772</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3574,21 +2920,6 @@
           <t>0.4836</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>0.2183</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>0.1996</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>0.2744</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3621,21 +2952,6 @@
           <t>0.2750</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>0.0427</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>0.0491</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>0.0610</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3668,21 +2984,6 @@
           <t>0.5935</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>0.0101</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>0.0124</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>0.0101</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3715,21 +3016,6 @@
           <t>0.7784</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>0.0506</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>0.0374</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>0.0745</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3762,21 +3048,6 @@
           <t>0.6050</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>0.1300</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>0.1316</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>0.2159</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3809,21 +3080,6 @@
           <t>0.8564</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>0.0713</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>0.0872</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>0.1475</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3856,21 +3112,6 @@
           <t>0.2327</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>0.1261</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>0.2097</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>0.2003</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3901,21 +3142,6 @@
       <c r="F18" t="inlineStr">
         <is>
           <t>0.6617</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>0.1695</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>0.1699</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>0.2152</t>
         </is>
       </c>
     </row>
@@ -3930,7 +3156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -4205,120 +3431,6 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>DINOv2</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>20</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>0.1837</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>0.1524</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>0.1203</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>0.0624</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>0.0205</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>OpenPhenom</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>20</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>0.1620</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>0.1326</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>0.1357</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>0.1003</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>0.0379</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>UNI</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>20</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>0.1994</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>0.1634</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>0.1284</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>0.0712</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>0.0216</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4330,7 +3442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4338,9 +3450,6 @@
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4369,21 +3478,6 @@
           <t>ResNet</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>DINOv2</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>OpenPhenom</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>UNI</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -4411,21 +3505,6 @@
           <t>0.6991</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>0.1006</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>0.1264</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>0.1430</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4453,21 +3532,6 @@
           <t>0.5520</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>0.0130</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>0.0139</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>0.0131</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -4495,21 +3559,6 @@
           <t>0.7772</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>0.0256</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>0.0240</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>0.0235</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4537,21 +3586,6 @@
           <t>0.7348</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>0.0392</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>0.0381</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>0.0392</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4579,21 +3613,6 @@
           <t>0.0836</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>0.0005</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>0.0006</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>0.0006</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4621,21 +3640,6 @@
           <t>0.5255</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>0.0463</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>0.0515</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>0.0611</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4663,21 +3667,6 @@
           <t>0.4743</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>0.0237</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>0.0214</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>0.0289</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4705,21 +3694,6 @@
           <t>0.8487</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>0.2260</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>0.2227</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>0.2546</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4747,21 +3721,6 @@
           <t>0.9213</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>0.2280</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>0.2013</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>0.2410</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4789,21 +3748,6 @@
           <t>0.7559</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>0.5340</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>0.4488</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>0.5436</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4831,21 +3775,6 @@
           <t>0.5876</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>0.2060</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>0.1686</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>0.2190</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -4873,21 +3802,6 @@
           <t>0.8247</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>0.3404</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>0.3296</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>0.3483</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4915,21 +3829,6 @@
           <t>0.1804</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>0.0044</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>0.0042</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>0.0039</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4957,21 +3856,6 @@
           <t>0.7860</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>0.2714</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>0.2421</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>0.2923</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -4999,21 +3883,6 @@
           <t>0.1679</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>0.0117</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>0.0106</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>0.0140</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5041,21 +3910,6 @@
           <t>0.2530</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>0.0508</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>0.0408</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>0.0607</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -5083,21 +3937,6 @@
           <t>0.7243</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>0.1965</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>0.1702</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>0.2078</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -5125,21 +3964,6 @@
           <t>0.8149</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>0.3016</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>0.2796</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>0.3113</t>
-        </is>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -5167,21 +3991,6 @@
           <t>0.7349</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>0.1888</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>0.1564</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>0.2165</t>
-        </is>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5207,21 +4016,6 @@
       <c r="E21" t="inlineStr">
         <is>
           <t>0.6024</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>0.1524</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>0.1326</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>0.1634</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ExprBaseline results for all datasets; document external model differences
- make_paper_excel.py: add KRONOS18/MIBI/IMC ExprBaseline from paper_clean
- CLAUDE.md: document KRONOS paper DINOv2/UNI/CA-MAE vs our implementation
- New tools: marker_attribution.py, cluster_attribution.py (IG-based cell type discovery)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/paper_results.xlsx
+++ b/paper_results.xlsx
@@ -1346,7 +1346,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -1621,6 +1621,48 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ExprBaseline</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>16</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>0.6249</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>0.6009</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>0.6298</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>0.5134</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>0.2610</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>0.0973</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1632,7 +1674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1640,7 +1682,8 @@
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1671,6 +1714,11 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>ExprBaseline</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>KRONOS</t>
         </is>
       </c>
@@ -1703,6 +1751,11 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>0.7190</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
           <t>0.7927</t>
         </is>
       </c>
@@ -1735,6 +1788,11 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
+          <t>0.7750</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
           <t>0.8369</t>
         </is>
       </c>
@@ -1767,6 +1825,11 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
+          <t>0.4574</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
           <t>0.9089</t>
         </is>
       </c>
@@ -1799,6 +1862,11 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>0.6450</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
           <t>0.6817</t>
         </is>
       </c>
@@ -1831,6 +1899,11 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
+          <t>0.8360</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
           <t>0.8473</t>
         </is>
       </c>
@@ -1863,6 +1936,11 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
+          <t>0.0585</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
           <t>0.6186</t>
         </is>
       </c>
@@ -1895,6 +1973,11 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
+          <t>0.8709</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
           <t>0.9053</t>
         </is>
       </c>
@@ -1927,6 +2010,11 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
+          <t>0.5145</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
           <t>0.5368</t>
         </is>
       </c>
@@ -1959,6 +2047,11 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
+          <t>0.7183</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
           <t>0.7317</t>
         </is>
       </c>
@@ -1991,6 +2084,11 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
+          <t>0.5932</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
           <t>0.8357</t>
         </is>
       </c>
@@ -2023,6 +2121,11 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
+          <t>0.4392</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
           <t>0.5737</t>
         </is>
       </c>
@@ -2055,6 +2158,11 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
+          <t>0.7149</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
           <t>0.7747</t>
         </is>
       </c>
@@ -2087,6 +2195,11 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
+          <t>0.7775</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
           <t>0.7505</t>
         </is>
       </c>
@@ -2119,6 +2232,11 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
+          <t>0.5911</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
           <t>0.6458</t>
         </is>
       </c>
@@ -2151,6 +2269,11 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
+          <t>0.4426</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
           <t>0.8150</t>
         </is>
       </c>
@@ -2183,6 +2306,11 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
+          <t>0.9236</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
           <t>0.9267</t>
         </is>
       </c>
@@ -2214,6 +2342,11 @@
         </is>
       </c>
       <c r="F18" t="inlineStr">
+        <is>
+          <t>0.6298</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
         <is>
           <t>0.7614</t>
         </is>
@@ -2516,32 +2649,32 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.7400</t>
+          <t>0.7042</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.7586</t>
+          <t>0.7542</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0.6617</t>
+          <t>0.6270</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0.5322</t>
+          <t>0.4629</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>0.2042</t>
+          <t>0.2216</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>0.0672</t>
+          <t>0.0949</t>
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
@@ -2629,7 +2762,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0.8812</t>
+          <t>0.8430</t>
         </is>
       </c>
     </row>
@@ -2661,7 +2794,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0.6105</t>
+          <t>0.5699</t>
         </is>
       </c>
     </row>
@@ -2693,7 +2826,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.8776</t>
+          <t>0.8493</t>
         </is>
       </c>
     </row>
@@ -2725,7 +2858,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0.9450</t>
+          <t>0.9373</t>
         </is>
       </c>
     </row>
@@ -2757,7 +2890,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0.7388</t>
+          <t>0.5742</t>
         </is>
       </c>
     </row>
@@ -2789,7 +2922,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>0.5026</t>
+          <t>0.4773</t>
         </is>
       </c>
     </row>
@@ -2821,7 +2954,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>0.3686</t>
+          <t>0.4387</t>
         </is>
       </c>
     </row>
@@ -2853,7 +2986,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>0.9819</t>
+          <t>0.9805</t>
         </is>
       </c>
     </row>
@@ -2885,7 +3018,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>0.8557</t>
+          <t>0.8269</t>
         </is>
       </c>
     </row>
@@ -2917,7 +3050,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>0.4836</t>
+          <t>0.4511</t>
         </is>
       </c>
     </row>
@@ -2949,7 +3082,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>0.2750</t>
+          <t>0.2852</t>
         </is>
       </c>
     </row>
@@ -2981,7 +3114,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>0.5935</t>
+          <t>0.5508</t>
         </is>
       </c>
     </row>
@@ -3013,7 +3146,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0.7784</t>
+          <t>0.7278</t>
         </is>
       </c>
     </row>
@@ -3045,7 +3178,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0.6050</t>
+          <t>0.5544</t>
         </is>
       </c>
     </row>
@@ -3077,7 +3210,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>0.8564</t>
+          <t>0.8359</t>
         </is>
       </c>
     </row>
@@ -3109,7 +3242,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>0.2327</t>
+          <t>0.1301</t>
         </is>
       </c>
     </row>
@@ -3141,7 +3274,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>0.6617</t>
+          <t>0.6270</t>
         </is>
       </c>
     </row>
@@ -3156,7 +3289,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -3431,6 +3564,48 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ExprBaseline</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>20</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>0.7072</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>0.7309</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>0.6579</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>0.6272</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>0.4221</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>0.2127</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3442,7 +3617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3450,6 +3625,7 @@
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3478,6 +3654,11 @@
           <t>ResNet</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>ExprBaseline</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3505,6 +3686,11 @@
           <t>0.6991</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0.7556</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3532,6 +3718,11 @@
           <t>0.5520</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0.6688</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3559,6 +3750,11 @@
           <t>0.7772</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>0.8275</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3586,6 +3782,11 @@
           <t>0.7348</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>0.7771</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3613,6 +3814,11 @@
           <t>0.0836</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>0.7887</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3640,6 +3846,11 @@
           <t>0.5255</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>0.5606</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3667,6 +3878,11 @@
           <t>0.4743</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>0.4662</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3694,6 +3910,11 @@
           <t>0.8487</t>
         </is>
       </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>0.8544</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3721,6 +3942,11 @@
           <t>0.9213</t>
         </is>
       </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>0.9332</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3748,6 +3974,11 @@
           <t>0.7559</t>
         </is>
       </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>0.7278</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3775,6 +4006,11 @@
           <t>0.5876</t>
         </is>
       </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>0.6237</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3802,6 +4038,11 @@
           <t>0.8247</t>
         </is>
       </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>0.8025</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3829,6 +4070,11 @@
           <t>0.1804</t>
         </is>
       </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>0.2355</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3856,6 +4102,11 @@
           <t>0.7860</t>
         </is>
       </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>0.7552</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3883,6 +4134,11 @@
           <t>0.1679</t>
         </is>
       </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>0.2201</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3910,6 +4166,11 @@
           <t>0.2530</t>
         </is>
       </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>0.3242</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3937,6 +4198,11 @@
           <t>0.7243</t>
         </is>
       </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>0.7852</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3964,6 +4230,11 @@
           <t>0.8149</t>
         </is>
       </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>0.8144</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3991,6 +4262,11 @@
           <t>0.7349</t>
         </is>
       </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>0.8333</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4016,6 +4292,11 @@
       <c r="E21" t="inlineStr">
         <is>
           <t>0.6024</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>0.6579</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ablation sheet to Excel; fix ExprBaseline cLISI/iLISI; patch LISI tool
- make_paper_excel.py: add Ablations sheet (3 groups, 13 variants + 2 repeats of baseline)
- make_paper_excel.py: switch CODEX_cHL ExprBaseline to paper_clean path (consistent with others)
- patch_lisi.py: tool to backfill cLISI/iLISI into ExprBaseline metrics.json from saved val_results.npz
- CODEX_cHL ExprBaseline rerun submitted (job 11814999) to paper_clean with val_results.npz saved

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/paper_results.xlsx
+++ b/paper_results.xlsx
@@ -15,6 +15,7 @@
     <sheet name="MIBI_TNBC_AP" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="IMC_NB_TumorSub" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="IMC_NB_TumorSub_AP" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Ablations" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -420,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -695,48 +696,6 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>ExprBaseline</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>16</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>0.6601</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>0.6298</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>0.6643</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>0.5111</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>0.2568</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>0.0901</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -748,7 +707,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -756,7 +715,6 @@
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -785,11 +743,6 @@
           <t>ResNet</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>ExprBaseline</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -817,11 +770,6 @@
           <t>0.7690</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>0.7392</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -849,11 +797,6 @@
           <t>0.7619</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>0.7947</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -881,11 +824,6 @@
           <t>0.8006</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>0.6531</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -913,11 +851,6 @@
           <t>0.6440</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>0.6365</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -945,11 +878,6 @@
           <t>0.7987</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>0.8461</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -977,11 +905,6 @@
           <t>0.0843</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>0.1006</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1009,11 +932,6 @@
           <t>0.6895</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>0.8761</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1041,11 +959,6 @@
           <t>0.5121</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>0.5342</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1073,11 +986,6 @@
           <t>0.6919</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>0.7291</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1105,11 +1013,6 @@
           <t>0.7555</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>0.8386</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1137,11 +1040,6 @@
           <t>0.3832</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>0.4506</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1169,11 +1067,6 @@
           <t>0.6033</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>0.6818</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1201,11 +1094,6 @@
           <t>0.7602</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>0.7838</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1233,11 +1121,6 @@
           <t>0.5205</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>0.6213</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1265,11 +1148,6 @@
           <t>0.4307</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>0.4184</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1297,11 +1175,6 @@
           <t>0.9185</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>0.9248</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1327,11 +1200,6 @@
       <c r="E18" t="inlineStr">
         <is>
           <t>0.6327</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>0.6643</t>
         </is>
       </c>
     </row>
@@ -2677,8 +2545,16 @@
           <t>0.0949</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>0.0676</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>0.0966</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3603,8 +3479,16 @@
           <t>0.2127</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>0.0432</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>0.1705</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4303,4 +4187,862 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Variant</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>LP Balanced Acc</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>LP Macro F1</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>LP mAP</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>kNN Balanced Acc</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>NMI</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>ARI</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>cLISI (norm)</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>iLISI (norm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Channel Aug</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Full aug (8k) ★</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>0.7123</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>0.6722</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>0.7179</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0.5909</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0.3077</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>0.1431</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>0.1008</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Channel Aug</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>No channel aug</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>0.7130</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>0.6600</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>0.7177</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0.5688</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0.2758</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>0.1353</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>0.1242</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Channel Aug</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>No channel drop</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>0.6953</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>0.6563</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>0.6971</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>0.5844</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>0.3071</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>0.1659</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>0.0960</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Channel Aug</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>No channel shift</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>0.7006</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>0.6668</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>0.7134</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>0.5914</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>0.3036</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>0.1436</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>0.0994</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Channel Aug</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>No noise</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>0.7236</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>0.6730</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>0.7328</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>0.5958</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>0.2874</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>0.1362</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>0.1060</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Channel Aug</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Drop p=0.05</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>0.7038</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>0.6657</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>0.7129</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>0.6016</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>0.3311</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>0.1745</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>0.0930</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Channel Aug</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Drop p=0.20</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>0.7262</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>0.6828</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>0.7358</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>0.5811</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>0.3005</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>0.1433</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>0.1074</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Training Length</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2k iters</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>0.7094</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>0.6682</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>0.7178</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>0.6024</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>0.3150</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>0.1531</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>0.0910</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Training Length</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>4k iters</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>0.7134</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>0.6728</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>0.7230</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>0.5975</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>0.3164</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>0.1515</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>0.0966</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Training Length</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Full aug (8k) ★</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>0.7123</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>0.6722</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>0.7179</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>0.5909</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>0.3077</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>0.1431</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>0.1008</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Model Capacity</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>4 mix blocks</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>0.7089</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>0.6702</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>0.7204</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>0.5911</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>0.3061</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>0.1408</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>0.1019</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Model Capacity</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Full aug (8k) ★</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>0.7123</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>0.6722</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>0.7179</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>0.5909</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>0.3077</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>0.1431</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>0.1008</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Model Capacity</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>12 mix blocks</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>0.7014</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>0.6649</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>0.7115</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>0.5918</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>0.3078</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>0.1533</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>0.1005</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Model Capacity</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>256 mix channels</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>0.6956</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>0.6545</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>0.7030</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>0.5913</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>0.3000</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>0.1453</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>0.1003</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Model Capacity</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>768 mix channels</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>0.7163</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>0.6773</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>0.7258</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>0.5925</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>0.3128</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>0.1601</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>0.0993</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Show mean±std for ExprBaseline CV results in Excel
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/paper_results.xlsx
+++ b/paper_results.xlsx
@@ -2517,42 +2517,42 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.7042</t>
+          <t>0.7042 ± 0.0174</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.7542</t>
+          <t>0.7542 ± 0.0214</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0.6270</t>
+          <t>0.6270 ± 0.0276</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0.4629</t>
+          <t>0.4629 ± 0.0190</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>0.2216</t>
+          <t>0.2216 ± 0.0444</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>0.0949</t>
+          <t>0.0949 ± 0.0264</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>0.0676</t>
+          <t>0.0676 ± 0.0088</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>0.0966</t>
+          <t>0.0966 ± 0.0358</t>
         </is>
       </c>
     </row>
@@ -3451,42 +3451,42 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.7072</t>
+          <t>0.7072 ± 0.0204</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.7309</t>
+          <t>0.7309 ± 0.0194</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0.6579</t>
+          <t>0.6579 ± 0.0048</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0.6272</t>
+          <t>0.6272 ± 0.0097</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>0.4221</t>
+          <t>0.4221 ± 0.0301</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>0.2127</t>
+          <t>0.2127 ± 0.0241</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>0.0432</t>
+          <t>0.0432 ± 0.0040</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>0.1705</t>
+          <t>0.1705 ± 0.0263</t>
         </is>
       </c>
     </row>

</xml_diff>